<commit_message>
Fix refund classification and update dashboard
</commit_message>
<xml_diff>
--- a/excel/household_financial_dashboard.xlsx
+++ b/excel/household_financial_dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jared/Desktop/household-financial-analysis/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F10C5F11-E2F4-044A-9785-DC94660B8FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37142525-F83B-D04E-94F1-67EF96A9A57E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="260" yWindow="500" windowWidth="28040" windowHeight="16940" xr2:uid="{20982C6F-3B99-E546-AC6C-61A1DEEF3B37}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -488,23 +488,23 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="44" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="44" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -609,15 +609,6 @@
       </font>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -635,6 +626,15 @@
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -664,171 +664,6 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>12700</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E920495F-1FCB-3C55-CB15-E5CB7F3FB39B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="12700" y="1422400"/>
-          <a:ext cx="5753100" cy="4292600"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>571500</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D7891CB9-5B38-B7A4-D760-1435D9AC619A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5956300" y="1422400"/>
-          <a:ext cx="5740400" cy="4292600"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>711200</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Picture 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85854C42-6AE6-4DEA-4417-49B02C7507F3}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11874500" y="1422400"/>
-          <a:ext cx="5753100" cy="4292600"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
       <xdr:colOff>25400</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
@@ -853,7 +688,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -908,7 +743,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -963,7 +798,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -1018,7 +853,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -1046,16 +881,181 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>393700</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{41391FF7-0603-AA7B-EA59-6643AD5A392A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25400" y="1485900"/>
+          <a:ext cx="5753100" cy="4292600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77514B23-6FAA-D823-F0AD-8A9BA369AD84}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5956300" y="1485900"/>
+          <a:ext cx="5740400" cy="4292600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>698500</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>673100</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6D6F9A9B-B9BF-C4D1-61B7-767EA0C21752}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11861800" y="1485900"/>
+          <a:ext cx="5753100" cy="4292600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9C21C3D2-6289-6B4C-95E8-DA2399312F39}" name="Table1" displayName="Table1" ref="A3:C12" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9C21C3D2-6289-6B4C-95E8-DA2399312F39}" name="Table1" displayName="Table1" ref="A3:C12" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A3:C12" xr:uid="{9C21C3D2-6289-6B4C-95E8-DA2399312F39}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{50BA5619-4628-8345-871A-9334F28576FA}" name="Category" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{502EA8C3-74BC-FF4F-A236-397DF2E41F34}" name="Annual Spending" dataDxfId="7" dataCellStyle="Currency"/>
-    <tableColumn id="3" xr3:uid="{48B2BAAA-85F3-BA44-8A22-F93AA059F60D}" name="% of total" dataDxfId="10" dataCellStyle="Percent">
+    <tableColumn id="1" xr3:uid="{50BA5619-4628-8345-871A-9334F28576FA}" name="Category" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{502EA8C3-74BC-FF4F-A236-397DF2E41F34}" name="Annual Spending" dataDxfId="8" dataCellStyle="Currency"/>
+    <tableColumn id="3" xr3:uid="{48B2BAAA-85F3-BA44-8A22-F93AA059F60D}" name="% of total" dataDxfId="7" dataCellStyle="Percent">
       <calculatedColumnFormula>B4/SUM($B$4:B$12)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1420,7 +1420,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27" x14ac:dyDescent="0.35">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="11" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1443,34 +1443,34 @@
       <c r="H3" s="15"/>
     </row>
     <row r="4" spans="1:8" ht="22" x14ac:dyDescent="0.3">
-      <c r="A4" s="14">
+      <c r="A4" s="16">
         <f>'Financial Health'!B4</f>
         <v>174923.04</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="11">
+      <c r="B4" s="16"/>
+      <c r="C4" s="17">
         <f>'Financial Health'!B5</f>
-        <v>371758.31999999995</v>
-      </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="13">
+        <v>372066.27</v>
+      </c>
+      <c r="D4" s="17"/>
+      <c r="E4" s="18">
         <f>'Financial Health'!B6</f>
-        <v>-196835.27999999994</v>
-      </c>
-      <c r="F4" s="13"/>
-      <c r="G4" s="12">
+        <v>-197143.23</v>
+      </c>
+      <c r="F4" s="18"/>
+      <c r="G4" s="19">
         <f>'Financial Health'!B10</f>
         <v>40</v>
       </c>
-      <c r="H4" s="12"/>
+      <c r="H4" s="19"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="G5" s="17" t="s">
+      <c r="G5" s="12" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="75" spans="6:6" ht="19" x14ac:dyDescent="0.25">
-      <c r="F75" s="19" t="s">
+      <c r="F75" s="14" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
     </row>
     <row r="77" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F77" s="18" t="s">
+      <c r="F77" s="13" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C4" s="3">
         <f>B4/SUM($B$4:B$12)</f>
-        <v>0.41397039883330661</v>
+        <v>0.41362776582784566</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1554,11 +1554,11 @@
         <v>5</v>
       </c>
       <c r="B5" s="4">
-        <v>57362.35</v>
+        <v>57670.3</v>
       </c>
       <c r="C5" s="3">
         <f>B5/SUM($B$4:B$12)</f>
-        <v>0.15430011088924656</v>
+        <v>0.1550000756585648</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="C6" s="3">
         <f>B6/SUM($B$4:B$12)</f>
-        <v>0.12228659737864106</v>
+        <v>0.12218538380272954</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="C7" s="3">
         <f>B7/SUM($B$4:B$12)</f>
-        <v>9.1995251108300702E-2</v>
+        <v>9.1919108926482362E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C8" s="3">
         <f>B8/SUM($B$4:B$12)</f>
-        <v>8.4844099790422997E-2</v>
+        <v>8.4773876438732271E-2</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="C9" s="3">
         <f>B9/SUM($B$4:B$12)</f>
-        <v>5.2086177923334719E-2</v>
+        <v>5.2043067489025548E-2</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="C10" s="3">
         <f>B10/SUM($B$4:B$12)</f>
-        <v>3.5378979547787931E-2</v>
+        <v>3.5349697246138435E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="C11" s="3">
         <f>B11/SUM($B$4:B$12)</f>
-        <v>3.1608411615374206E-2</v>
+        <v>3.1582250119044655E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="C12" s="3">
         <f>B12/SUM($B$4:B$12)</f>
-        <v>1.3529972913585367E-2</v>
+        <v>1.3518774491436699E-2</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -1664,11 +1664,11 @@
         <v>15</v>
       </c>
       <c r="B16" s="6">
-        <v>29194.28</v>
+        <v>29213.26</v>
       </c>
       <c r="C16" s="1">
         <f>(B16-$B$29)/$B$29</f>
-        <v>-5.7636800166301648E-2</v>
+        <v>-5.7804621741175219E-2</v>
       </c>
       <c r="D16" t="str">
         <f>IF(C16&gt;=10%, "High", "Normal")</f>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="C17" s="1">
         <f t="shared" ref="C17:C27" si="0">(B17-$B$29)/$B$29</f>
-        <v>-2.4234131464764542E-2</v>
+        <v>-2.5041748611073895E-2</v>
       </c>
       <c r="D17" t="str">
         <f t="shared" ref="D17:D27" si="1">IF(C17&gt;=10%, "High", "Normal")</f>
@@ -1696,11 +1696,11 @@
         <v>17</v>
       </c>
       <c r="B18" s="6">
-        <v>34800.93</v>
+        <v>34878.800000000003</v>
       </c>
       <c r="C18" s="1">
         <f t="shared" si="0"/>
-        <v>0.12334045408855945</v>
+        <v>0.1249221812017523</v>
       </c>
       <c r="D18" t="str">
         <f t="shared" si="1"/>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="C19" s="1">
         <f t="shared" si="0"/>
-        <v>-4.9474077674979834E-2</v>
+        <v>-5.0260804345419297E-2</v>
       </c>
       <c r="D19" t="str">
         <f t="shared" si="1"/>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="C20" s="1">
         <f t="shared" si="0"/>
-        <v>-7.0565199455388181E-2</v>
+        <v>-7.1334469528774994E-2</v>
       </c>
       <c r="D20" t="str">
         <f t="shared" si="1"/>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="C21" s="1">
         <f t="shared" si="0"/>
-        <v>-6.9274038036324431E-3</v>
+        <v>-7.7493452980834472E-3</v>
       </c>
       <c r="D21" t="str">
         <f t="shared" si="1"/>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="C22" s="1">
         <f t="shared" si="0"/>
-        <v>-0.12732271869530729</v>
+        <v>-0.12804501198133325</v>
       </c>
       <c r="D22" t="str">
         <f t="shared" si="1"/>
@@ -1776,11 +1776,11 @@
         <v>22</v>
       </c>
       <c r="B23" s="6">
-        <v>33698.04</v>
+        <v>33842.35</v>
       </c>
       <c r="C23" s="1">
         <f t="shared" si="0"/>
-        <v>8.7740228651775706E-2</v>
+        <v>9.1494265255488066E-2</v>
       </c>
       <c r="D23" t="str">
         <f t="shared" si="1"/>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="C24" s="1">
         <f t="shared" si="0"/>
-        <v>-2.4441362872524353E-2</v>
+        <v>-2.5248808498550455E-2</v>
       </c>
       <c r="D24" t="str">
         <f t="shared" si="1"/>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="C25" s="1">
         <f t="shared" si="0"/>
-        <v>0.10964381375512994</v>
+        <v>0.10872538916252759</v>
       </c>
       <c r="D25" t="str">
         <f t="shared" si="1"/>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="C26" s="1">
         <f t="shared" si="0"/>
-        <v>7.5090720229207299E-3</v>
+        <v>6.6751818164008086E-3</v>
       </c>
       <c r="D26" t="str">
         <f t="shared" si="1"/>
@@ -1840,11 +1840,11 @@
         <v>26</v>
       </c>
       <c r="B27" s="6">
-        <v>31982.62</v>
+        <v>32049.41</v>
       </c>
       <c r="C27" s="1">
         <f t="shared" si="0"/>
-        <v>3.2368125614512085E-2</v>
+        <v>3.3667792568243433E-2</v>
       </c>
       <c r="D27" t="str">
         <f t="shared" si="1"/>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="B29" s="6">
         <f>AVERAGE(B16:B27)</f>
-        <v>30979.86</v>
+        <v>31005.522499999995</v>
       </c>
     </row>
   </sheetData>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B5" s="8">
         <f>SUM('Spending Summary'!B4:B12)</f>
-        <v>371758.31999999995</v>
+        <v>372066.27</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="B6" s="9">
         <f>B4-B5</f>
-        <v>-196835.27999999994</v>
+        <v>-197143.23</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="B7" s="1">
         <f>B6/B4</f>
-        <v>-1.1252678892386041</v>
+        <v>-1.1270283777368608</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>